<commit_message>
Se suben datos hasta jun-2026 y se hacen las transformaciones correspondientes a las variables para que sean estacionarias
</commit_message>
<xml_diff>
--- a/input/INDPRO.xlsx
+++ b/input/INDPRO.xlsx
@@ -32,7 +32,7 @@
     <t>This data may be copyrighted. Please refer to the Terms of Use: https://fred.stlouisfed.org/legal#fred-terms-faq</t>
   </si>
   <si>
-    <t>File Created: 2026-03-24 1:36 am CDT</t>
+    <t>File Created: 2026-08-10 11:59 am CDT</t>
   </si>
   <si>
     <t>INDPRO</t>
@@ -41,7 +41,7 @@
     <t>Industrial Production: Total Index, Index 2017=100, Monthly, Seasonally Adjusted</t>
   </si>
   <si>
-    <t>Data Updated: 2026-03-16</t>
+    <t>Data Updated: 2026-07-17</t>
   </si>
   <si>
     <t>observation_date</t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1287"/>
+  <dimension ref="A1:B1291"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -10735,7 +10735,7 @@
         <v>45931</v>
       </c>
       <c r="B1283" s="2">
-        <v>101.2075</v>
+        <v>101.2195</v>
       </c>
     </row>
     <row r="1284" spans="1:2">
@@ -10743,7 +10743,7 @@
         <v>45962</v>
       </c>
       <c r="B1284" s="2">
-        <v>101.3605</v>
+        <v>101.0344</v>
       </c>
     </row>
     <row r="1285" spans="1:2">
@@ -10751,7 +10751,7 @@
         <v>45992</v>
       </c>
       <c r="B1285" s="2">
-        <v>101.6781</v>
+        <v>101.4941</v>
       </c>
     </row>
     <row r="1286" spans="1:2">
@@ -10759,7 +10759,7 @@
         <v>46023</v>
       </c>
       <c r="B1286" s="2">
-        <v>102.3963</v>
+        <v>101.0388</v>
       </c>
     </row>
     <row r="1287" spans="1:2">
@@ -10767,7 +10767,39 @@
         <v>46054</v>
       </c>
       <c r="B1287" s="2">
-        <v>102.551</v>
+        <v>101.9263</v>
+      </c>
+    </row>
+    <row r="1288" spans="1:2">
+      <c r="A1288" s="4">
+        <v>46082</v>
+      </c>
+      <c r="B1288" s="2">
+        <v>101.6172</v>
+      </c>
+    </row>
+    <row r="1289" spans="1:2">
+      <c r="A1289" s="4">
+        <v>46113</v>
+      </c>
+      <c r="B1289" s="2">
+        <v>102.4196</v>
+      </c>
+    </row>
+    <row r="1290" spans="1:2">
+      <c r="A1290" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B1290" s="2">
+        <v>102.5606</v>
+      </c>
+    </row>
+    <row r="1291" spans="1:2">
+      <c r="A1291" s="4">
+        <v>46174</v>
+      </c>
+      <c r="B1291" s="2">
+        <v>102.6395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>